<commit_message>
Updating pipeline for historical bronze
</commit_message>
<xml_diff>
--- a/documentation/workflow/historical_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/historical_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F83E95-B7E0-6140-9092-EB5EE32619C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821EC2BA-D57A-834C-9955-4569A573C1A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="77">
   <si>
     <t>PaymentTerms</t>
   </si>
@@ -216,9 +216,6 @@
   </si>
   <si>
     <t>originating_company,  postingdate</t>
-  </si>
-  <si>
-    <t>originating_company, itemcategorycode</t>
   </si>
   <si>
     <t>originating_company, postingdate</t>
@@ -1029,10 +1026,10 @@
         <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -1049,10 +1046,10 @@
         <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1069,10 +1066,10 @@
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -1080,16 +1077,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D15" t="s">
         <v>48</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F15" t="s">
         <v>58</v>
@@ -1109,10 +1106,10 @@
         <v>29</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1123,7 +1120,7 @@
         <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D17" t="s">
         <v>48</v>
@@ -1132,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -1149,10 +1146,10 @@
         <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="18" x14ac:dyDescent="0.2">
@@ -1163,13 +1160,13 @@
         <v>22</v>
       </c>
       <c r="C19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D19" t="s">
         <v>48</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F19" t="s">
         <v>58</v>
@@ -1189,7 +1186,7 @@
         <v>29</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F20" t="s">
         <v>58</v>
@@ -1200,16 +1197,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" t="s">
         <v>76</v>
-      </c>
-      <c r="C21" t="s">
-        <v>77</v>
       </c>
       <c r="D21" t="s">
         <v>48</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
         <v>58</v>
@@ -1232,7 +1229,7 @@
         <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1252,7 +1249,7 @@
         <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to historical workflow
</commit_message>
<xml_diff>
--- a/documentation/workflow/historical_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/historical_bronze_workflow_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE850E5-9645-FB4A-A7EF-50473696580B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B017958-5603-1445-BB82-D7F4418C17FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
+    <workbookView minimized="1" xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
   </bookViews>
   <sheets>
     <sheet name="Historical" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="74">
   <si>
     <t>PaymentTerms</t>
   </si>
@@ -328,6 +328,12 @@
   </si>
   <si>
     <t>documentno</t>
+  </si>
+  <si>
+    <t>FundingBody</t>
+  </si>
+  <si>
+    <t>phoneno, address</t>
   </si>
 </sst>
 </file>
@@ -772,7 +778,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBA92A4A-7349-FF40-A839-841302118E9B}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
@@ -1237,6 +1243,26 @@
         <v>60</v>
       </c>
     </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
update to historical bronze workflow
</commit_message>
<xml_diff>
--- a/documentation/workflow/historical_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/historical_bronze_workflow_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E3F55A-45CB-4A4A-9250-C9E178DCBE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB708B09-0DC1-264B-A3DD-1E14747FA592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
+    <workbookView xWindow="700" yWindow="500" windowWidth="28100" windowHeight="17500" xr2:uid="{63FD3DF8-BE3E-CA4B-9FF3-647869DC2764}"/>
   </bookViews>
   <sheets>
     <sheet name="Historical" sheetId="2" r:id="rId1"/>
@@ -206,9 +206,6 @@
     <t>documenttype, vendorno,  buyfromvendorno, globaldimension1code, globaldimension2code, purchasercode, sourcecode, balaccounttype</t>
   </si>
   <si>
-    <t>city, postcode, globaldimension1code, globaldimension2code, customerpostinggroup, customerpricegroup, languagecode, paymenttermscode, salespersoncode, shipmentmethodcode, shippingagentcode,  customerdiscgroup, countryregioncode,  billtocustomerno, locationcode, contacttype</t>
-  </si>
-  <si>
     <t>originating_company</t>
   </si>
   <si>
@@ -222,47 +219,6 @@
   </si>
   <si>
     <t xml:space="preserve">selltocustomerno, billtocustomerno, billtocity,  billtocontact, shiptocity,  shiptocontact, paymenttermscode,  shipmentmethodcode,  locationcode, shortcutdimension1code, shortcutdimension2code, customerpostinggroup,  currencycode,  salespersoncode, orderno,  genbuspostinggroup, vatcountryregioncode, transactiontype, transportmethod,  selltocity, billtopostcode, billtocounty, billtocountryregioncode, selltopostcode,  selltocounty,  shiptopostcode, shiptocounty,  shiptocountryregioncode, balaccounttype,  paymentmethodcode, shippingagentcode,  preassignedno, sourcecode,  vatbuspostinggroup,  prepaymentorderno,  dimensionsetid,  custledgerentryno, selltocontactno, billtocontactno </t>
-  </si>
-  <si>
-    <r>
-      <t>selltocustomerno,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Menlo"/>
-        <family val="2"/>
-      </rPr>
-      <t>no</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Menlo"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Menlo"/>
-        <family val="2"/>
-      </rPr>
-      <t>type</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Menlo"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, locationcode, postinggroup, unitofmeasure, shortcutdimension1code, shortcutdimension2code, customerpricegroup, orderno, jobno, shipmentno, billtocustomerno, genbuspostinggroup, genprodpostinggroup, vatcalculationtype, transactiontype, taxcategory, vatbuspostinggroup, vatprodpostinggroup, vatidentifier </t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">buyfromvendorno, paytovendorno, paytocity, paytocontact, shiptocode, shiptocity, shiptocountryregioncode, paymenttermscode, shipmentmethodcode, locationcode, shortcutdimension1code, shortcutdimension2code, vendorpostinggroup , currencycode, invoicedisccode, languagecode, purchasercode, orderno, vendorinvoiceno, selltocustomerno, reasoncode, genbuspostinggroup, transactiontype, transportmethod, vatcountryregioncode, buyfromcity, buyfromcontact, paytopostcode, paytocounty, paytocountryregioncode, buyfrompostcode, buyfromcounty, buyfromcountryregioncode, shiptopostcode, shiptocounty, shiptocountryregioncode, balaccounttype, paymentmethodcode, preassignedno, sourcecode, vatbuspostinggroup, prepaymentorderno, quoteno, creditorno, dimensionsetid, remittocode, vendorledgerentryno, buyfromcontactno, paytocontactno, responsibilitycenter, pricecalculationmethod </t>
@@ -325,6 +281,50 @@
   </si>
   <si>
     <t>phoneno, address</t>
+  </si>
+  <si>
+    <r>
+      <t>selltocustomerno,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>no</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t>type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Menlo"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, locationcode, postinggroup, unitofmeasure, shortcutdimension1code, shortcutdimension2code, customerpricegroup, orderno, jobno, shipmentno, billtocustomerno, genbuspostinggroup, genprodpostinggroup, vatcalculationtype, transactiontype, taxcategory, vatbuspostinggroup, vatprodpostinggroup, vatidentifier, funder </t>
+    </r>
+  </si>
+  <si>
+    <t>city, postcode, globaldimension1code, globaldimension2code, customerpostinggroup, customerpricegroup, languagecode, paymenttermscode, salespersoncode, shipmentmethodcode, shippingagentcode,  customerdiscgroup, countryregioncode,  billtocustomerno, locationcode, contacttype,customertype</t>
   </si>
 </sst>
 </file>
@@ -851,7 +851,7 @@
         <v>45</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -871,7 +871,7 @@
         <v>46</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -891,7 +891,7 @@
         <v>51</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -911,7 +911,7 @@
         <v>52</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -928,10 +928,10 @@
         <v>26</v>
       </c>
       <c r="E8" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -951,7 +951,7 @@
         <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -971,7 +971,7 @@
         <v>54</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -991,7 +991,7 @@
         <v>55</v>
       </c>
       <c r="F11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -1008,10 +1008,10 @@
         <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -1028,10 +1028,10 @@
         <v>35</v>
       </c>
       <c r="E13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1048,10 +1048,10 @@
         <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -1059,19 +1059,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
         <v>47</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -1088,10 +1088,10 @@
         <v>28</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1099,10 +1099,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D17" t="s">
         <v>47</v>
@@ -1111,7 +1111,7 @@
         <v>39</v>
       </c>
       <c r="F17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -1128,10 +1128,10 @@
         <v>28</v>
       </c>
       <c r="E18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="18" x14ac:dyDescent="0.2">
@@ -1139,19 +1139,19 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D19" t="s">
         <v>47</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="F19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="18" x14ac:dyDescent="0.2">
@@ -1168,10 +1168,10 @@
         <v>28</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="18" x14ac:dyDescent="0.2">
@@ -1179,19 +1179,19 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D21" t="s">
         <v>47</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1211,7 +1211,7 @@
         <v>38</v>
       </c>
       <c r="F22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1231,12 +1231,12 @@
         <v>38</v>
       </c>
       <c r="F23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
         <v>21</v>
@@ -1245,13 +1245,13 @@
         <v>32</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E24" t="s">
         <v>38</v>
       </c>
       <c r="F24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>